<commit_message>
fix(s1): short situation choice and direct S6–S12 route; subcontractor/customer roles (#269)
Detailed 16-question check becomes optional (S1); S0 is a short choice of
six situations with an explicit start step and path. Overdue payment goes
S6→S12 without S2–S5, including unreconciled balances via the settlement
register. Buyer files name the parties Субподрядчик and Заказчик; the oral
agreement sentence is replaced with the approved wording. Five new checks
fail on the previous candidate and pass here; LibreOffice layer reports
ПРОПУСК when only libreoffice-core is installed.

BUILD CANDIDATE / NO PUBLIC LAUNCH. LEGAL_REVIEW_REQUIRED unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UmCUuQToGDpJHXok26LuA6
</commit_message>
<xml_diff>
--- a/tools/candidates/s1-oplata-za-raboty/02-pervichnaya-proverka-i-kontrol.xlsx
+++ b/tools/candidates/s1-oplata-za-raboty/02-pervichnaya-proverka-i-kontrol.xlsx
@@ -488,14 +488,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Первичная проверка и маршрутизация</t>
+          <t>Детальная проверка — по желанию</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ответьте на каждый вопрос: Да / Нет / Не знаю. Итог и следующий шаг считаются автоматически. Жёлтые ячейки — ввод.</t>
+          <t>Необязательно. Ситуация выбирается в файле 01, таблица 1. Эта проверка — для случая, когда вы сомневаетесь в выборе: ответьте на вопросы Да / Нет / Не знаю, итог покажет ситуацию или границу. Строку «Последний день срока оплаты» ниже заполняйте в любом случае (шаг 6). Жёлтые ячейки — ввод.</t>
         </is>
       </c>
     </row>
@@ -549,7 +549,7 @@
       <c r="C6" s="5" t="n"/>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Нет → шаги 2–5</t>
+          <t>Нет → шаги 2–5 (ситуация Г)</t>
         </is>
       </c>
     </row>
@@ -629,7 +629,7 @@
       <c r="C11" s="5" t="n"/>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Да → шаг 5</t>
+          <t>Да → шаг 5 (ситуация Д)</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       <c r="C19" s="5" t="n"/>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Нет → шаг 6</t>
+          <t>Нет → шаг 6 (ситуация Б)</t>
         </is>
       </c>
     </row>
@@ -773,7 +773,7 @@
       <c r="C20" s="5" t="n"/>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Нет → шаг 4</t>
+          <t>Нет → шаг 4 (ситуация Е)</t>
         </is>
       </c>
     </row>
@@ -5100,12 +5100,12 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Ответьте на все вопросы</t>
+          <t>Проверка не пройдена</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Заполните колонку «Ответ» во всех строках.</t>
+          <t>Проверка по желанию. Для итога ответьте на все вопросы; без неё выберите ситуацию в файле 01, таблица 1.</t>
         </is>
       </c>
     </row>
@@ -5219,12 +5219,12 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>ШАГИ 2–5: оформить и сдать работы</t>
+          <t>СИТУАЦИЯ Г, ШАГ 2: оформить и сдать работы</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Оформите акты (файлы 04–07), проверьте (09), передайте с доказательством и закройте замечания (10).</t>
+          <t>Оформите акты (файлы 04–07), проверьте (09), передайте с доказательством и закройте замечания (10), затем шаг 6.</t>
         </is>
       </c>
     </row>
@@ -5258,7 +5258,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Доведите до конца шаги 2–5 и сверку (шаг 6). Вернитесь к маршруту на следующий день после истечения срока.</t>
+          <t>Маршрут начните на следующий день после срока. До этого документы можно готовить по ситуации Г (шаги 2–5).</t>
         </is>
       </c>
     </row>
@@ -5270,7 +5270,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>ШАГ 4: подтвердить передачу</t>
+          <t>СИТУАЦИЯ Е, ШАГ 4: подтвердить передачу</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -5287,7 +5287,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>ШАГ 5: закрыть замечания</t>
+          <t>СИТУАЦИЯ Д, ШАГ 5: закрыть замечания</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -5304,12 +5304,12 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>ШАГ 6: подтвердить сумму</t>
+          <t>СИТУАЦИЯ Б, ШАГ 6: подтвердить сумму</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Заполните реестр взаиморасчётов (файл 08) и предложите заказчику акт сверки.</t>
+          <t>Заполните реестр взаиморасчётов (файл 08) и предложите заказчику акт сверки; шаги 2–5 не нужны.</t>
         </is>
       </c>
     </row>
@@ -5326,7 +5326,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Шаг 6 → шаг 7: зафиксируйте долг и дату начала просрочки, затем переговоры (файл 11).</t>
+          <t>Ситуация А: шаги 6–12. Зафиксируйте долг и дату начала просрочки, затем переговоры (файл 11).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
wip: preserve S1 financial implementation state
</commit_message>
<xml_diff>
--- a/tools/candidates/s1-oplata-za-raboty/02-pervichnaya-proverka-i-kontrol.xlsx
+++ b/tools/candidates/s1-oplata-za-raboty/02-pervichnaya-proverka-i-kontrol.xlsx
@@ -824,7 +824,7 @@
     <row r="27" ht="45" customHeight="1">
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Последний день срока оплаты (по договору или двустороннему соглашению; если он пришёлся на нерабочий день — ближайший следующий рабочий день, ст. 193 ГК РФ)</t>
+          <t>Последний день срока оплаты (по договору или двустороннему соглашению; если он пришёлся на нерабочий день — ближайший следующий рабочий день, ст. 193 ГК РФ). Если актов несколько и сроки оплаты по ним разные, заполните срок по каждому акту в файле 08, лист «Долг по актам»: эта строка тогда служит для самого раннего акта</t>
         </is>
       </c>
       <c r="C27" s="8" t="n"/>
@@ -832,7 +832,7 @@
     <row r="28" ht="45" customHeight="1">
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Первый день просрочки (перенесите в файл 14, лист «Ввод»)</t>
+          <t>Первый день просрочки (по каждому акту он свой: файл 08, лист «Долг по актам», оттуда — в файл 14, лист «Акты», вместе с долгом на первый день просрочки)</t>
         </is>
       </c>
       <c r="C28" s="9">

</xml_diff>